<commit_message>
Added more context for HIGHEST and HIGH priority
</commit_message>
<xml_diff>
--- a/SIMAP-Model-Analysis/Olga's proposal.xlsx
+++ b/SIMAP-Model-Analysis/Olga's proposal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\ietf\Misc\SIMAP-Model-Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A754E440-799D-4750-A37E-43D7F5759362}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E558E576-DAAC-487A-AD49-47D043573A2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-1545" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="41">
   <si>
     <t>Requirement</t>
   </si>
@@ -59,9 +59,6 @@
       </rPr>
       <t>“It is possible for links at one level of a hierarchy to map to multiple links at another level of the hierarchy.  For example, a VPN topology might model VPN tunnels as links.  Where a VPN tunnel maps to a path that is composed of a chain of several links, the link will contain a list of those supporting links.  Likewise, it is possible for a link at one level of a hierarchy to aggregate a bundle of links at another level of the hierarchy. "</t>
     </r>
-  </si>
-  <si>
-    <t>Use RFC8345 and when needed augment the fields that we identified are needed.</t>
   </si>
   <si>
     <t>We followed the RFC8345 approach and did the same in Hackathons and PoC for L2/L3/ISIS/OSPF/BGP/MPLS-TE/MPLS-LDP/SRv6/L3VPN. We modelled all layers, including tunnels and paths using the basic IETF approach. We identified some additional fields that are needed for supporting relations to add semantics, but we determined that all topological layers and entities can be modelled via the RFC8345 entities and relations and that these fields can be added via just adding fields to RFC8345 entities and relations.
@@ -150,13 +147,7 @@
     <t xml:space="preserve">HIGH </t>
   </si>
   <si>
-    <t>RFC8345 implements it via generic approach, every layer uses the same core entities that can be augmented for specific layer/technology.</t>
-  </si>
-  <si>
     <t>RFC8345 implements it via supporting relations: supporting-network (underlay network), supporting-node, supporting-link, supporting-termination-point. Using RFC8345 would require to navigate via supporting relation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">We need to be able to add any additional semantic (primary/backup, hub/spoke, uni/nni, …) </t>
   </si>
   <si>
     <t xml:space="preserve">RFC8345 Gap.
@@ -166,6 +157,229 @@
     <t>RFC8345 Gap.
 RFC8345 only supports supporting between the same types of entities (network-&gt;supporting-&gt;networ, node-&gt;supporting-&gt;node, termination-point-&gt;supporting-&gt;termination-point, link-&gt;supporting-&gt;link).
 The requirement cannot be supported by RFC8345.</t>
+  </si>
+  <si>
+    <t>Req No</t>
+  </si>
+  <si>
+    <t>RFC8345 implements it via generic approach and the network can have either one or multiple network-types that can identify the layers.</t>
+  </si>
+  <si>
+    <t>Use RFC8345 and augment the fields (not entities) that we identified are needed. We can augment network, node, termination-point, link and supporting relations with a dditional attributes, but all topological entities should be modelled using the 4 core concepts: network, node, termination-point and link at any layer, including tunnels and paths.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">RFC8345 already supports the flexibility to to support both the same network topology instance with multiple layers (e.g., Layer 2 and Layer 3) or separate network topology instances with supporting relations between them (e.g., separate Layer 2 and Layer 3). Multiple topology layers can  be grouped into the same network topology instance, if solution requires.
+Some improvements can </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>OPTIONALLY</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> be done via REQ-SEMANTIC to
+1) add some hierarchy to layers via sublayers (e.g. layer tunnel, with tunnel and path as sublayers)
+2) allow the individual nodes, tps, links to belong to separate layers or sublayers when  network has multiple layers (network types). This would allow that we have 1 instance of network/nodes for both tunnels and paths with just links at different layers/sub-layers)
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">No model changes mandatory, same as in 1.
+Network-types for sublayers can be </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>OPTIONALLY</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> added but that is not priority in making decision about the approach. The current model is sufficient to support the requirements.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">RFC8345 approach is sufficient for the requirements. 
+It may </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>OPTIONALLY</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> be improved with sublayers (e.g. tunnel layer with tunnel and path sublayers) and allowing that individual links/tps belong to only 1 sublayer/layers out of multiple ones defined for the network.</t>
+    </r>
+  </si>
+  <si>
+    <t>We used supporting relation from RFC8345 to navigate all layers from the service to the physical, including tunnels and paths. We identified some additional meta data required to understand the layering using supporting relation and would suggest the solution in REQ-SEMANTICS.
+When there are multiple tunnels or paths, RFC8345 does not have semantics. We identified required extensions in the hackathon where we modellled SRv6 with all layers from service to physical, including policies, paths, segment lists and segments.</t>
+  </si>
+  <si>
+    <t>RFC8345 approach is sufficient to navigate, additional semantics would be proposed in REQ-SEMANTIC.</t>
+  </si>
+  <si>
+    <t>We need to be able to add any additional semantic (primary/backup, hub/spoke, uni/nni, …) . 
+We focused on this requirement in IETF124 Hackathon:
+1. We tried to compute the physical path of a packet based on an SRv6 SIMAP model
+2.We analyzed what extensions are needed for the SIMAP model based on RFC8345 to support path computation and identified that the following is needed for supporting relation for links: order, preference, weight</t>
+  </si>
+  <si>
+    <t>Option 3: Generic way for any extensions via extensions attributes (via anydata to support completely unstructured data)
+Apply this grouping to every major entity in the topology model and in supporting relations.
+     grouping simap-common {
+       description "A reusable set of optional extensions for network,
+                    node, termination point and link";
+       :
+       :
+       anydata extension {
+         description
+           "The extension point for any other meta info or data or any
+           unknown extensions. Proposed solution for SIMAP requirement
+           REQ-EXTENSIBLE. Any additional info that is topologically
+           significant can also be added this way for requirement
+           REQ-SEMANTIC or REQ-PROPERTIES.";
+       }
+     }</t>
+  </si>
+  <si>
+    <t>No model changes mandatory to to basic navigation for current tunnels/paths, but additional semantics required to understand supporting relations meaning for multiple tunnels and paths configured/used. 
+We identified order, preference and weight as important meta data that needs to be added - proposal in REQ-SEMANTIC.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">
+Option 1: Specific solution for supporting links relations
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+  augment "/nw:networks/nw:network/nt:link/nt:supporting-link" {
+    description
+      "Add semantics for supporting link selection and ordering.";
+    leaf link-status {
+      type enumeration {
+        enum current {
+          description "This is the active supporting link currently in use.";
+        }
+        enum alternative {
+          description "This is a backup or standby supporting link.";
+        }
+      }
+      description "Indicates if the supporting link is current or an alternative.";
+    }
+    leaf order {
+      type uint32;
+      description
+        "The numeric order of the supporting link within the list.";
+    }
+    leaf preference {
+      type uint32;
+      description
+        "The preference value for selecting this link. 
+         Higher values typically indicate higher preference.";
+    }
+    leaf weight {
+      type uint32;
+      description
+        "The weight associated with this link, often used for 
+         load-balancing or cost calculations.";
+    }
+  }
+}
+</t>
+    </r>
+  </si>
+  <si>
+    <t>Option 2: Generic way for any extensions via extensions attributes (via identityref)
+Apply this grouping to every major entity in the topology model and in supporting relations.
+grouping generic-attributes {
+  list attribute {
+    key "name";
+    leaf name {
+      type identityref {
+        base attribute-type;
+      }
+    }
+    leaf value {
+      type string;
+      description "The value of the attribute, typically string-encoded.";
+    }
+  }
+}
+identity attribute-type {
+  description "Base identity for all generic attributes.";
+}
+identity link-supporting-attribute-type {
+  base attribute-type;
+  description "Base identity for all link supporting attribute types";
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Although we identified the attributes needed for this case, some other attributes may be needed based on other use cases. 
+Therefore there are 2 approaches: either add exact attributes to the supporting relation via augmentation or reuse the generic approach for REQ-EXTENSION to enable any extension.
+There are pros and cons of each approach, and the target model can support all 3. For attributes that we know based on hackathons and product experience, we can use Option1, for any future ones we can allow extensions via Option 2/3.
+Alternatively, we can go with Option 2 for any RFC8345 attribute extensions, with additional fields that can identify all required meta data for the attributes. </t>
+  </si>
+  <si>
+    <t>Our requirement from the modelling exercise / PoCs / Hackathon is that we had some TPs at higher layers that do not have supporting relation to TPs at the lower layer and the only way to be able to navigate supporting dependencies top to bottom (or for assurance bottom to top) was to add supporting relation to node at the lower layer. Examples: loopback is at Layer 3, but does not have Layer 2 or Physical TP for supporting. We also have in PoC one type of SID (that we modelled as TPs) at SRv6 layer that did not have any TPs as supporting, so we needed to build relation to the Node at the layer below.
+There was also requirement that Italo had to have supporting between a node and a network.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Augment RFC8345 nodes and termination-points to support the new supporting relations.</t>
+  </si>
+  <si>
+    <t>augment "/nw:networks/nw:network/nw:node/nt:termination-point" {
+  container supporting-node {
+    leaf network-ref {
+      type leafref {
+        path "/nw:networks/nw:network/nw:network-id";
+      }
+    }
+    leaf node-ref {
+      type leafref {
+        path "/nw:networks/nw:network[nw:network-id=current()/../network-ref]"
+           + "/nw:node/nw:node-id";
+      }
+    }
+    description
+      "Identifies the specific node that supports this termination point.";
+  }
+}</t>
   </si>
 </sst>
 </file>
@@ -233,7 +447,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -248,6 +462,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -587,377 +807,230 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="28.9140625" customWidth="1"/>
-    <col min="2" max="2" width="35.83203125" customWidth="1"/>
-    <col min="3" max="4" width="49.83203125" customWidth="1"/>
-    <col min="5" max="5" width="32.33203125" customWidth="1"/>
-    <col min="6" max="6" width="113.9140625" customWidth="1"/>
+    <col min="2" max="2" width="28.9140625" customWidth="1"/>
+    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="4" max="5" width="49.83203125" customWidth="1"/>
+    <col min="6" max="6" width="32.33203125" customWidth="1"/>
+    <col min="7" max="7" width="73.33203125" customWidth="1"/>
+    <col min="8" max="8" width="81.9140625" customWidth="1"/>
+    <col min="9" max="9" width="79.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>16</v>
-      </c>
       <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="2"/>
+    <row r="2" spans="1:9">
+      <c r="A2" s="1"/>
       <c r="B2" s="2"/>
-      <c r="C2" s="1"/>
+      <c r="C2" s="2"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
     </row>
-    <row r="3" spans="1:6" ht="409.5" customHeight="1">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:9" ht="409.5" customHeight="1">
+      <c r="A3" s="1">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="321.5" customHeight="1">
+      <c r="A4" s="1">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="C4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>28</v>
+      </c>
     </row>
-    <row r="4" spans="1:6" ht="42">
-      <c r="A4" s="1" t="s">
+    <row r="5" spans="1:9" ht="165" customHeight="1">
+      <c r="A5" s="1">
+        <v>3</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="409.5" customHeight="1">
+      <c r="A6" s="1">
+        <v>4</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
+      <c r="E6" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>33</v>
+      </c>
     </row>
-    <row r="5" spans="1:6" ht="56">
-      <c r="A5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="1" t="s">
+    <row r="7" spans="1:9" ht="196">
+      <c r="A7" s="1">
+        <v>5</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
+      <c r="E7" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>40</v>
+      </c>
     </row>
-    <row r="6" spans="1:6" ht="41" customHeight="1">
-      <c r="A6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-    </row>
-    <row r="7" spans="1:6" ht="98">
-      <c r="A7" s="1" t="s">
+    <row r="8" spans="1:9">
+      <c r="A8" s="1">
+        <v>6</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="1"/>
+      <c r="C8" s="1" t="s">
+        <v>16</v>
+      </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
     </row>
-    <row r="9" spans="1:6">
-      <c r="A9" s="1" t="s">
-        <v>15</v>
+    <row r="9" spans="1:9">
+      <c r="A9" s="1">
+        <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="1"/>
+        <v>14</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>16</v>
+      </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
     </row>
-    <row r="10" spans="1:6">
-      <c r="A10" s="1" t="s">
-        <v>18</v>
+    <row r="10" spans="1:9">
+      <c r="A10" s="1">
+        <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="1"/>
+      <c r="C10" s="1" t="s">
+        <v>16</v>
+      </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
     </row>
-    <row r="11" spans="1:6">
-      <c r="A11" s="1" t="s">
-        <v>19</v>
+    <row r="11" spans="1:9">
+      <c r="A11" s="1">
+        <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="1"/>
+        <v>18</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>16</v>
+      </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-    </row>
-    <row r="13" spans="1:6">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-    </row>
-    <row r="17" spans="1:6">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-    </row>
-    <row r="18" spans="1:6">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-    </row>
-    <row r="19" spans="1:6">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-    </row>
-    <row r="21" spans="1:6">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-    </row>
-    <row r="22" spans="1:6">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-    </row>
-    <row r="23" spans="1:6">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-    </row>
-    <row r="24" spans="1:6">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-    </row>
-    <row r="25" spans="1:6">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
-    </row>
-    <row r="26" spans="1:6">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
-    </row>
-    <row r="27" spans="1:6">
-      <c r="A27" s="1"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
-      <c r="F27" s="1"/>
-    </row>
-    <row r="28" spans="1:6">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
-      <c r="F28" s="1"/>
-    </row>
-    <row r="29" spans="1:6">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-    </row>
-    <row r="30" spans="1:6">
-      <c r="A30" s="1"/>
-      <c r="B30" s="1"/>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
-    </row>
-    <row r="31" spans="1:6">
-      <c r="A31" s="1"/>
-      <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
-      <c r="D31" s="1"/>
-      <c r="E31" s="1"/>
-      <c r="F31" s="1"/>
-    </row>
-    <row r="32" spans="1:6">
-      <c r="A32" s="1"/>
-      <c r="B32" s="1"/>
-      <c r="C32" s="1"/>
-      <c r="D32" s="1"/>
-      <c r="E32" s="1"/>
-      <c r="F32" s="1"/>
-    </row>
-    <row r="33" spans="1:6">
-      <c r="A33" s="1"/>
-      <c r="B33" s="1"/>
-      <c r="C33" s="1"/>
-      <c r="D33" s="1"/>
-      <c r="E33" s="1"/>
-      <c r="F33" s="1"/>
-    </row>
-    <row r="34" spans="1:6">
-      <c r="A34" s="1"/>
-      <c r="B34" s="1"/>
-      <c r="C34" s="1"/>
-      <c r="D34" s="1"/>
-      <c r="E34" s="1"/>
-      <c r="F34" s="1"/>
-    </row>
-    <row r="35" spans="1:6">
-      <c r="A35" s="1"/>
-      <c r="B35" s="1"/>
-      <c r="C35" s="1"/>
-      <c r="D35" s="1"/>
-      <c r="E35" s="1"/>
-      <c r="F35" s="1"/>
-    </row>
-    <row r="36" spans="1:6">
-      <c r="A36" s="1"/>
-      <c r="B36" s="1"/>
-      <c r="C36" s="1"/>
-      <c r="D36" s="1"/>
-      <c r="E36" s="1"/>
-      <c r="F36" s="1"/>
-    </row>
-    <row r="37" spans="1:6">
-      <c r="A37" s="1"/>
-      <c r="B37" s="1"/>
-      <c r="C37" s="1"/>
-      <c r="D37" s="1"/>
-      <c r="E37" s="1"/>
-      <c r="F37" s="1"/>
+      <c r="G11" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="0" type="noConversion"/>

</xml_diff>